<commit_message>
update perhitungan dgn parameter dinamis
</commit_message>
<xml_diff>
--- a/data/file/tabel_IGSYC.xlsx
+++ b/data/file/tabel_IGSYC.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aryax punya\2026\KKA VAB\Aplikasi\imbalan-pasca-kerja-app\data\file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Kerjaan Arya\KKA VAB\Aplikasi\imbalan-pasca-kerja-app\data\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84EBBF8-EAF8-40D5-9D24-1F744FA6DEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25F5095B-9AAD-4ECC-B276-7EF6A9D0F227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{13D302E8-A00F-41E5-906F-072FF2494F16}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{13D302E8-A00F-41E5-906F-072FF2494F16}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="IBPA" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -89,6 +89,85 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{464271EF-B7B0-4297-B5F5-B325E1EC533E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3048000" y="0"/>
+          <a:ext cx="10744200" cy="5324475"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a14:hiddenLine>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -389,9 +468,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D4B26EF-FE81-4E19-AD0A-2E2FC440C7F4}">
   <dimension ref="A1:B63"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -399,7 +478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -407,7 +486,7 @@
         <v>4.4800000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0.5</v>
       </c>
@@ -415,7 +494,7 @@
         <v>4.4800000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -423,7 +502,7 @@
         <v>4.8099999999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1.5</v>
       </c>
@@ -431,7 +510,7 @@
         <v>4.8099999999999996</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -439,7 +518,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2.5</v>
       </c>
@@ -447,7 +526,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
@@ -455,7 +534,7 @@
         <v>5.33</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3.5</v>
       </c>
@@ -463,7 +542,7 @@
         <v>5.33</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -471,7 +550,7 @@
         <v>5.52</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>4.5</v>
       </c>
@@ -479,7 +558,7 @@
         <v>5.52</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5</v>
       </c>
@@ -487,7 +566,7 @@
         <v>5.67</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5.5</v>
       </c>
@@ -495,7 +574,7 @@
         <v>5.67</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>6</v>
       </c>
@@ -503,7 +582,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>6.5</v>
       </c>
@@ -511,7 +590,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>7</v>
       </c>
@@ -519,7 +598,7 @@
         <v>5.92</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>7.5</v>
       </c>
@@ -527,7 +606,7 @@
         <v>5.92</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>8</v>
       </c>
@@ -535,7 +614,7 @@
         <v>6.01</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>8.5</v>
       </c>
@@ -543,7 +622,7 @@
         <v>6.01</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>9</v>
       </c>
@@ -551,7 +630,7 @@
         <v>6.09</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>9.5</v>
       </c>
@@ -559,7 +638,7 @@
         <v>6.09</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>10</v>
       </c>
@@ -567,7 +646,7 @@
         <v>6.16</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>10.5</v>
       </c>
@@ -575,7 +654,7 @@
         <v>6.16</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>11</v>
       </c>
@@ -583,7 +662,7 @@
         <v>6.23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>11.5</v>
       </c>
@@ -591,7 +670,7 @@
         <v>6.23</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>12</v>
       </c>
@@ -599,7 +678,7 @@
         <v>6.28</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>12.5</v>
       </c>
@@ -607,7 +686,7 @@
         <v>6.28</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>13</v>
       </c>
@@ -615,7 +694,7 @@
         <v>6.33</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>13.5</v>
       </c>
@@ -623,7 +702,7 @@
         <v>6.33</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>14</v>
       </c>
@@ -631,7 +710,7 @@
         <v>6.37</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>14.5</v>
       </c>
@@ -639,7 +718,7 @@
         <v>6.37</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>15</v>
       </c>
@@ -647,7 +726,7 @@
         <v>6.41</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>15.5</v>
       </c>
@@ -655,7 +734,7 @@
         <v>6.41</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>16</v>
       </c>
@@ -663,7 +742,7 @@
         <v>6.45</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>16.5</v>
       </c>
@@ -671,7 +750,7 @@
         <v>6.45</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>17</v>
       </c>
@@ -679,7 +758,7 @@
         <v>6.48</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>17.5</v>
       </c>
@@ -687,7 +766,7 @@
         <v>6.48</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>18</v>
       </c>
@@ -695,7 +774,7 @@
         <v>6.51</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>18.5</v>
       </c>
@@ -703,7 +782,7 @@
         <v>6.51</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>19</v>
       </c>
@@ -711,7 +790,7 @@
         <v>6.54</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>19.5</v>
       </c>
@@ -719,7 +798,7 @@
         <v>6.54</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>20</v>
       </c>
@@ -727,7 +806,7 @@
         <v>6.56</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>20.5</v>
       </c>
@@ -735,7 +814,7 @@
         <v>6.56</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>21</v>
       </c>
@@ -743,7 +822,7 @@
         <v>6.58</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>21.5</v>
       </c>
@@ -751,7 +830,7 @@
         <v>6.58</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>22</v>
       </c>
@@ -759,7 +838,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>22.5</v>
       </c>
@@ -767,7 +846,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>23</v>
       </c>
@@ -775,7 +854,7 @@
         <v>6.62</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>23.5</v>
       </c>
@@ -783,7 +862,7 @@
         <v>6.62</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>24</v>
       </c>
@@ -791,7 +870,7 @@
         <v>6.63</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>24.5</v>
       </c>
@@ -799,7 +878,7 @@
         <v>6.63</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>25</v>
       </c>
@@ -807,7 +886,7 @@
         <v>6.64</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>25.5</v>
       </c>
@@ -815,7 +894,7 @@
         <v>6.64</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>26</v>
       </c>
@@ -823,7 +902,7 @@
         <v>6.66</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>26.5</v>
       </c>
@@ -831,7 +910,7 @@
         <v>6.66</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>27</v>
       </c>
@@ -839,7 +918,7 @@
         <v>6.67</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>27.5</v>
       </c>
@@ -847,7 +926,7 @@
         <v>6.67</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>28</v>
       </c>
@@ -855,7 +934,7 @@
         <v>6.68</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>28.5</v>
       </c>
@@ -863,7 +942,7 @@
         <v>6.68</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>29</v>
       </c>
@@ -871,7 +950,7 @@
         <v>6.68</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>29.5</v>
       </c>
@@ -879,7 +958,7 @@
         <v>6.68</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>30</v>
       </c>
@@ -887,7 +966,7 @@
         <v>6.69</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>30.5</v>
       </c>
@@ -897,5 +976,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>